<commit_message>
Add comprehensive tests for KPost API workflows
- Implement feature flow tests for the KPost Dashboard, ensuring consistency between homeDashboardMsgs and katchupDashboardMsg.
- Add tests for Katchup needs-id reads, documenting known gaps and blockers in the API.
- Create plain read tests for Katchup, covering various endpoints including unopened messages and search functionalities.
- Introduce device/security endpoint tests for the Profile module, explicitly skipping tests that cannot be run live due to architectural constraints.
- Add plain read tests for Profile, validating user details, digital cards, and language retrieval.
- Implement personalization tests for font and theme settings, ensuring changes persist and are accurately reflected in the database.
</commit_message>
<xml_diff>
--- a/KPOST API (6).xlsx
+++ b/KPOST API (6).xlsx
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2290" uniqueCount="1156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2290" uniqueCount="1157">
   <si>
     <t>https://kmail5.kpostindia.com/kmail5/v2/</t>
   </si>
@@ -1166,8 +1166,7 @@
 }</t>
   </si>
   <si>
-    <t>https://devapi2.kpostindia.com/v2/profile/fetchUserDetails/
-https://devapi2.kpostindia.com/v2/signupLogin/fetchUserDetails/</t>
+    <t>https://devapi2.kpostindia.com/v2/signupLogin/fetchUserDetails/</t>
   </si>
   <si>
     <t>0-SENTLETTERS_NOT_OPENED, 1-REPLY_NOT_RECEIVED, 2-REPLY_NOT_SENT</t>
@@ -23887,6 +23886,9 @@
   </si>
   <si>
     <t>.168.1.94</t>
+  </si>
+  <si>
+    <t>GET METHOD</t>
   </si>
 </sst>
 </file>
@@ -25525,7 +25527,7 @@
         <v>43</v>
       </c>
       <c r="L2" s="46" t="s">
-        <v>44</v>
+        <v>1156</v>
       </c>
       <c r="M2" s="48" t="s">
         <v>46</v>

</xml_diff>